<commit_message>
UG Excel Agenda 2026-2027
</commit_message>
<xml_diff>
--- a/inputs/UG Excel Agenda.xlsx
+++ b/inputs/UG Excel Agenda.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jspenc35\projects\curriculog_excel_sheet_generator\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37A9AE0F-FB78-4DDB-92F4-0A2B814BCEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D799D8-BA07-4C46-AF69-27769CD0E42D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="620" yWindow="900" windowWidth="21600" windowHeight="11180" xr2:uid="{125E1219-2066-4676-87E7-42C796F6CDDF}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{125E1219-2066-4676-87E7-42C796F6CDDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -567,7 +567,7 @@
     <t>UG Curriculum Committee</t>
   </si>
   <si>
-    <t>2025-2026 UG Add Course; 2025-2026 UG Revise Course; 2025-2026 UG Revise Program; 2025-2026 UG Add Program; 2025-2026 UG Change Course Number / Subject / Department; 2025-2026 UG Change Program Name / Department; 2025-2026 UG Drop/Archive Course; 2025-2026 UG End Program; Other Form; New Prefix/Subject Code (Undergraduate); Update Approval Tree(s) / Update Originator(s); Agenda Form - Administrative Use Only (Impact Sorting); New Degree Code; Informational Items; EL Designated Courses Reassessment; Courses Not Taught in 4 Years; Committee Reports; Content and Text Change (Non-Program Requirements); Correction Items</t>
+    <t xml:space="preserve">2025-2026 UG Add Course; 2025-2026 UG Revise Course; 2025-2026 UG Revise Program; 2025-2026 UG Add Program; 2025-2026 UG Change Course Number / Subject / Department; 2025-2026 UG Change Program Name / Department; 2025-2026 UG Drop/Archive Course; 2025-2026 UG End Program; Other Form; New Prefix/Subject Code (Undergraduate); Update Approval Tree(s) / Update Originator(s); Agenda Form - Administrative Use Only (Impact Sorting); New Degree Code; Informational Items; EL Designated Courses Reassessment; Courses Not Taught in 4 Years; Committee Reports; Content and Text Change (Non-Program Requirements); Correction Items; Agenda Form - Administrative Use Only; Committee Reports; New Degree Code; New, Rename, Move, or Drop Academic Unit; UG Content and Text Change; UG Informational Items; UG New Prefix/Subject Code; UG Other Form; 2026-2027 UG Add Course; 2026-2027 UG Drop/Archive Course; 2026-2027 UG Revise Course; 2026-2027 UG Revise Course (Dynamic Changes); 2026-2027 UG Add Program; 2026-2027 UG End Program; 2026-2027 UG Revise Program; 2026-2027 UG Revise Program (Dynamic Changes); </t>
   </si>
 </sst>
 </file>
@@ -1142,7 +1142,7 @@
         <v>18</v>
       </c>
       <c r="C4" s="8">
-        <v>45722</v>
+        <v>45884</v>
       </c>
       <c r="E4" s="8" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Look for proposal action, not action
</commit_message>
<xml_diff>
--- a/inputs/UG Excel Agenda.xlsx
+++ b/inputs/UG Excel Agenda.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jspenc35\projects\curriculog_excel_sheet_generator\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9A008B-6791-474A-9722-03D6D53F8DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801C609F-B7E7-430C-84BA-0F72F217AA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{125E1219-2066-4676-87E7-42C796F6CDDF}"/>
+    <workbookView xWindow="3030" yWindow="3030" windowWidth="21600" windowHeight="11295" xr2:uid="{125E1219-2066-4676-87E7-42C796F6CDDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="178">
   <si>
     <t>Field</t>
   </si>
@@ -567,7 +567,10 @@
     <t>UG Curriculum Committee</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-2026 UG Add Course; 2025-2026 UG Revise Course; 2025-2026 UG Revise Program; 2025-2026 UG Add Program; 2025-2026 UG Change Course Number / Subject / Department; 2025-2026 UG Change Program Name / Department; 2025-2026 UG Drop/Archive Course; 2025-2026 UG End Program; Other Form; New Prefix/Subject Code (Undergraduate); Update Approval Tree(s) / Update Originator(s); Agenda Form - Administrative Use Only (Impact Sorting); New Degree Code; Informational Items; EL Designated Courses Reassessment; Courses Not Taught in 4 Years; Committee Reports; Content and Text Change (Non-Program Requirements); Correction Items; Agenda Form - Administrative Use Only; Committee Reports; New Degree Code; New, Rename, Move, or Drop Academic Unit; UG Content and Text Change; UG Informational Items; UG New Prefix/Subject Code; UG Other Form; 2026-2027 UG Add Course; 2026-2027 UG Drop/Archive Course; 2026-2027 UG Revise Course; 2026-2027 UG Revise Course (Dynamic Changes); 2026-2027 UG Add Program; 2026-2027 UG End Program; 2026-2027 UG Revise Program; 2026-2027 UG Revise Program (Dynamic Changes); </t>
+    <t>2027-2028 UG Add Course; 2027-2028 UG Revise Course; 2027-2028 UG Revise Program; 2027-2028 UG Add Program; 2027-2028 UG Revise Course (Dynamic Changes); 2027-2028 UG Revise Program (Dynamic Changes); 2027-2028 UG Drop/Archive Course; 2027-2028 UG End Program; UG Other Form; UG New Prefix/Subject Code; UG Update Approver(s) / Update Originator(s); UG Agenda Form - Administrative Use Only; UG Amendment Form - Administrative Use Only; UG Informational Items; EL Designated Courses Reassessment; UG Courses Not Taught in 4 Years; Committee Reports; UG Content and Text Change; Correction Items; UG Academic Unit Changes; UG Reactivate Course</t>
+  </si>
+  <si>
+    <t>Proposal Action</t>
   </si>
 </sst>
 </file>
@@ -652,7 +655,7 @@
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1064,7 +1067,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="228.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="126.140625" style="8" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" style="8" customWidth="1"/>
     <col min="5" max="5" width="16.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -1106,9 +1109,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>177</v>
       </c>
       <c r="B2" t="s">
         <v>21</v>
@@ -1142,7 +1145,7 @@
         <v>18</v>
       </c>
       <c r="C4" s="8">
-        <v>45932</v>
+        <v>46280</v>
       </c>
       <c r="E4" s="8" t="b">
         <v>1</v>
@@ -1234,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A8F092-27DE-412E-8E0F-037E456B2861}">
-  <dimension ref="A1:E153"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="94.7109375" style="3" customWidth="1"/>
@@ -2045,6 +2048,11 @@
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
         <v>162</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154" s="3" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>